<commit_message>
feat: generate Hoenn region documentation spreadsheets
Adds script-generated Excel files detailing routes, spawns, challenge requirements, and Pokémon evolution paths for Hoenn (Region 3). Also adds a secondary map spots document.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/3_Hoenn_Data.xlsx
+++ b/3_Hoenn_Data.xlsx
@@ -483,7 +483,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>Challenge 1</v>
       </c>
       <c r="B5" t="str">
         <v>Route 103</v>
@@ -503,7 +503,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>Challenge 1</v>
       </c>
       <c r="B6" t="str">
         <v>Route 103</v>
@@ -523,7 +523,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>Challenge 1</v>
       </c>
       <c r="B7" t="str">
         <v>Route 103</v>
@@ -543,7 +543,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>Challenge 1</v>
       </c>
       <c r="B8" t="str">
         <v>Route 103</v>
@@ -563,7 +563,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>Challenge 1</v>
       </c>
       <c r="B9" t="str">
         <v>Route 103</v>
@@ -583,7 +583,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>Challenge 2</v>
       </c>
       <c r="B10" t="str">
         <v>Route 102</v>
@@ -603,7 +603,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>Challenge 2</v>
       </c>
       <c r="B11" t="str">
         <v>Route 102</v>
@@ -623,7 +623,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>Challenge 2</v>
       </c>
       <c r="B12" t="str">
         <v>Route 102</v>
@@ -643,7 +643,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>Challenge 2</v>
       </c>
       <c r="B13" t="str">
         <v>Route 102</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>Challenge 2</v>
       </c>
       <c r="B14" t="str">
         <v>Route 102</v>
@@ -683,7 +683,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v/>
+        <v>Challenge 2</v>
       </c>
       <c r="B15" t="str">
         <v>Route 102</v>
@@ -703,7 +703,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>Challenge 3</v>
       </c>
       <c r="B16" t="str">
         <v>Route 104</v>
@@ -723,7 +723,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>Challenge 3</v>
       </c>
       <c r="B17" t="str">
         <v>Route 104</v>
@@ -743,7 +743,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>Challenge 3</v>
       </c>
       <c r="B18" t="str">
         <v>Route 104</v>
@@ -763,7 +763,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>Challenge 3</v>
       </c>
       <c r="B19" t="str">
         <v>Route 104</v>
@@ -783,7 +783,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>Challenge 3</v>
       </c>
       <c r="B20" t="str">
         <v>Route 104</v>
@@ -803,7 +803,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>Challenge 4</v>
       </c>
       <c r="B21" t="str">
         <v>Petalburg Woods</v>
@@ -823,7 +823,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>Challenge 4</v>
       </c>
       <c r="B22" t="str">
         <v>Petalburg Woods</v>
@@ -843,7 +843,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v/>
+        <v>Challenge 4</v>
       </c>
       <c r="B23" t="str">
         <v>Petalburg Woods</v>
@@ -863,7 +863,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v/>
+        <v>Challenge 4</v>
       </c>
       <c r="B24" t="str">
         <v>Petalburg Woods</v>
@@ -883,7 +883,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>Challenge 4</v>
       </c>
       <c r="B25" t="str">
         <v>Petalburg Woods</v>
@@ -903,7 +903,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v>Challenge 4</v>
       </c>
       <c r="B26" t="str">
         <v>Petalburg Woods</v>
@@ -923,7 +923,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>Challenge 5</v>
       </c>
       <c r="B27" t="str">
         <v>Route 116</v>
@@ -943,7 +943,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
+        <v>Challenge 5</v>
       </c>
       <c r="B28" t="str">
         <v>Route 116</v>
@@ -963,7 +963,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>Challenge 5</v>
       </c>
       <c r="B29" t="str">
         <v>Route 116</v>
@@ -983,7 +983,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
+        <v>Challenge 5</v>
       </c>
       <c r="B30" t="str">
         <v>Route 116</v>
@@ -1003,7 +1003,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>Challenge 5</v>
       </c>
       <c r="B31" t="str">
         <v>Route 116</v>
@@ -1023,7 +1023,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B32" t="str">
         <v>Granite Cave</v>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B33" t="str">
         <v>Granite Cave</v>
@@ -1063,7 +1063,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B34" t="str">
         <v>Granite Cave</v>
@@ -1083,7 +1083,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B35" t="str">
         <v>Granite Cave</v>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B36" t="str">
         <v>Granite Cave</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B37" t="str">
         <v>Granite Cave</v>
@@ -1143,7 +1143,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B38" t="str">
         <v>Granite Cave</v>
@@ -1163,7 +1163,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v/>
+        <v>Challenge 7</v>
       </c>
       <c r="B39" t="str">
         <v>Granite Cave</v>
@@ -1183,7 +1183,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v/>
+        <v>Challenge 8</v>
       </c>
       <c r="B40" t="str">
         <v>Tiny Fishing Spot</v>
@@ -1203,7 +1203,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v/>
+        <v>Challenge 8</v>
       </c>
       <c r="B41" t="str">
         <v>Tiny Fishing Spot</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v/>
+        <v>Challenge 8</v>
       </c>
       <c r="B42" t="str">
         <v>Tiny Fishing Spot</v>
@@ -1243,7 +1243,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v/>
+        <v>Challenge 8</v>
       </c>
       <c r="B43" t="str">
         <v>Tiny Fishing Spot</v>
@@ -1263,7 +1263,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
+        <v>Challenge 10</v>
       </c>
       <c r="B44" t="str">
         <v>Route 107</v>
@@ -1283,7 +1283,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v/>
+        <v>Challenge 10</v>
       </c>
       <c r="B45" t="str">
         <v>Route 107</v>
@@ -1303,7 +1303,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v/>
+        <v>Challenge 10</v>
       </c>
       <c r="B46" t="str">
         <v>Route 107</v>
@@ -1323,7 +1323,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B47" t="str">
         <v>Route 110</v>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B48" t="str">
         <v>Route 110</v>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B49" t="str">
         <v>Route 110</v>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B50" t="str">
         <v>Route 110</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B51" t="str">
         <v>Route 110</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B52" t="str">
         <v>Route 110</v>
@@ -1443,7 +1443,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v/>
+        <v>Challenge 12</v>
       </c>
       <c r="B53" t="str">
         <v>Route 110</v>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B54" t="str">
         <v>Route 117</v>
@@ -1483,7 +1483,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B55" t="str">
         <v>Route 117</v>
@@ -1503,7 +1503,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B56" t="str">
         <v>Route 117</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B57" t="str">
         <v>Route 117</v>
@@ -1543,7 +1543,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B58" t="str">
         <v>Route 117</v>
@@ -1563,7 +1563,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B59" t="str">
         <v>Route 117</v>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v/>
+        <v>Challenge 13</v>
       </c>
       <c r="B60" t="str">
         <v>Route 117</v>
@@ -1603,7 +1603,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v/>
+        <v>Challenge 14</v>
       </c>
       <c r="B61" t="str">
         <v>Route 111</v>
@@ -1623,7 +1623,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v/>
+        <v>Challenge 14</v>
       </c>
       <c r="B62" t="str">
         <v>Route 111</v>
@@ -1643,7 +1643,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v/>
+        <v>Challenge 14</v>
       </c>
       <c r="B63" t="str">
         <v>Route 111</v>
@@ -1663,7 +1663,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v/>
+        <v>Challenge 14</v>
       </c>
       <c r="B64" t="str">
         <v>Route 111</v>
@@ -1683,7 +1683,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v/>
+        <v>Challenge 14</v>
       </c>
       <c r="B65" t="str">
         <v>Route 111</v>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v/>
+        <v>Challenge 16</v>
       </c>
       <c r="B66" t="str">
         <v>Fiery Path</v>
@@ -1723,7 +1723,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v/>
+        <v>Challenge 16</v>
       </c>
       <c r="B67" t="str">
         <v>Fiery Path</v>
@@ -1743,7 +1743,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v/>
+        <v>Challenge 16</v>
       </c>
       <c r="B68" t="str">
         <v>Fiery Path</v>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v/>
+        <v>Challenge 16</v>
       </c>
       <c r="B69" t="str">
         <v>Fiery Path</v>
@@ -1783,7 +1783,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v/>
+        <v>Challenge 16</v>
       </c>
       <c r="B70" t="str">
         <v>Fiery Path</v>
@@ -1803,7 +1803,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v/>
+        <v>Challenge 16</v>
       </c>
       <c r="B71" t="str">
         <v>Fiery Path</v>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v/>
+        <v>Challenge 17</v>
       </c>
       <c r="B72" t="str">
         <v>Jagged Pass</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v/>
+        <v>Challenge 17</v>
       </c>
       <c r="B73" t="str">
         <v>Jagged Pass</v>
@@ -1863,7 +1863,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v/>
+        <v>Challenge 17</v>
       </c>
       <c r="B74" t="str">
         <v>Jagged Pass</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v/>
+        <v>Challenge 18</v>
       </c>
       <c r="B75" t="str">
         <v>Route 113</v>
@@ -1903,7 +1903,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v/>
+        <v>Challenge 18</v>
       </c>
       <c r="B76" t="str">
         <v>Route 113</v>
@@ -1923,7 +1923,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v/>
+        <v>Challenge 18</v>
       </c>
       <c r="B77" t="str">
         <v>Route 113</v>
@@ -1943,7 +1943,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B78" t="str">
         <v>Route 114</v>
@@ -1963,7 +1963,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B79" t="str">
         <v>Route 114</v>
@@ -1983,7 +1983,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B80" t="str">
         <v>Route 114</v>
@@ -2003,7 +2003,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B81" t="str">
         <v>Route 114</v>
@@ -2023,7 +2023,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B82" t="str">
         <v>Route 114</v>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B83" t="str">
         <v>Route 114</v>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v/>
+        <v>Challenge 19</v>
       </c>
       <c r="B84" t="str">
         <v>Route 114</v>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v/>
+        <v>Challenge 20</v>
       </c>
       <c r="B85" t="str">
         <v>Meteor Falls</v>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v/>
+        <v>Challenge 20</v>
       </c>
       <c r="B86" t="str">
         <v>Meteor Falls</v>
@@ -2123,7 +2123,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v/>
+        <v>Challenge 20</v>
       </c>
       <c r="B87" t="str">
         <v>Meteor Falls</v>
@@ -2143,7 +2143,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v/>
+        <v>Challenge 20</v>
       </c>
       <c r="B88" t="str">
         <v>Meteor Falls</v>
@@ -2163,7 +2163,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v/>
+        <v>Challenge 20</v>
       </c>
       <c r="B89" t="str">
         <v>Meteor Falls</v>
@@ -2183,7 +2183,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v/>
+        <v>Challenge 21</v>
       </c>
       <c r="B90" t="str">
         <v>Route 115</v>
@@ -2203,7 +2203,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v/>
+        <v>Challenge 21</v>
       </c>
       <c r="B91" t="str">
         <v>Route 115</v>
@@ -2223,7 +2223,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v/>
+        <v>Challenge 21</v>
       </c>
       <c r="B92" t="str">
         <v>Route 115</v>
@@ -2243,7 +2243,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v/>
+        <v>Challenge 21</v>
       </c>
       <c r="B93" t="str">
         <v>Route 115</v>
@@ -2263,7 +2263,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v/>
+        <v>Challenge 21</v>
       </c>
       <c r="B94" t="str">
         <v>Route 115</v>
@@ -2283,7 +2283,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v/>
+        <v>Challenge 23</v>
       </c>
       <c r="B95" t="str">
         <v>Route 118</v>
@@ -2303,7 +2303,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v/>
+        <v>Challenge 23</v>
       </c>
       <c r="B96" t="str">
         <v>Route 118</v>
@@ -2323,7 +2323,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v/>
+        <v>Challenge 23</v>
       </c>
       <c r="B97" t="str">
         <v>Route 118</v>
@@ -2343,7 +2343,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v/>
+        <v>Challenge 23</v>
       </c>
       <c r="B98" t="str">
         <v>Route 118</v>
@@ -2363,7 +2363,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v/>
+        <v>Challenge 23</v>
       </c>
       <c r="B99" t="str">
         <v>Route 118</v>
@@ -2383,7 +2383,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v/>
+        <v>Challenge 23</v>
       </c>
       <c r="B100" t="str">
         <v>Route 118</v>
@@ -2403,7 +2403,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v/>
+        <v>Challenge 24</v>
       </c>
       <c r="B101" t="str">
         <v>Small Fishing Spot</v>
@@ -2423,7 +2423,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v/>
+        <v>Challenge 24</v>
       </c>
       <c r="B102" t="str">
         <v>Small Fishing Spot</v>
@@ -2443,7 +2443,7 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v/>
+        <v>Challenge 24</v>
       </c>
       <c r="B103" t="str">
         <v>Small Fishing Spot</v>
@@ -2463,7 +2463,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v/>
+        <v>Challenge 24</v>
       </c>
       <c r="B104" t="str">
         <v>Small Fishing Spot</v>
@@ -2483,7 +2483,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v/>
+        <v>Challenge 24</v>
       </c>
       <c r="B105" t="str">
         <v>Small Fishing Spot</v>
@@ -2503,7 +2503,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v/>
+        <v>Challenge 24</v>
       </c>
       <c r="B106" t="str">
         <v>Small Fishing Spot</v>
@@ -2523,7 +2523,7 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v/>
+        <v>Challenge 25</v>
       </c>
       <c r="B107" t="str">
         <v>Route 119</v>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v/>
+        <v>Challenge 25</v>
       </c>
       <c r="B108" t="str">
         <v>Route 119</v>
@@ -2563,7 +2563,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v/>
+        <v>Challenge 25</v>
       </c>
       <c r="B109" t="str">
         <v>Route 119</v>
@@ -2583,7 +2583,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v/>
+        <v>Challenge 25</v>
       </c>
       <c r="B110" t="str">
         <v>Route 119</v>
@@ -2603,7 +2603,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v/>
+        <v>Challenge 25</v>
       </c>
       <c r="B111" t="str">
         <v>Route 119</v>
@@ -2623,7 +2623,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v/>
+        <v>Challenge 25</v>
       </c>
       <c r="B112" t="str">
         <v>Route 119</v>
@@ -2643,7 +2643,7 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B113" t="str">
         <v>Route 120</v>
@@ -2663,7 +2663,7 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B114" t="str">
         <v>Route 120</v>
@@ -2683,7 +2683,7 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B115" t="str">
         <v>Route 120</v>
@@ -2703,7 +2703,7 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B116" t="str">
         <v>Route 120</v>
@@ -2723,7 +2723,7 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B117" t="str">
         <v>Route 120</v>
@@ -2743,7 +2743,7 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B118" t="str">
         <v>Route 120</v>
@@ -2763,7 +2763,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v/>
+        <v>Challenge 26</v>
       </c>
       <c r="B119" t="str">
         <v>Route 120</v>
@@ -2783,7 +2783,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v/>
+        <v>Challenge 27</v>
       </c>
       <c r="B120" t="str">
         <v>Route 121</v>
@@ -2803,7 +2803,7 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v/>
+        <v>Challenge 27</v>
       </c>
       <c r="B121" t="str">
         <v>Route 121</v>
@@ -2823,7 +2823,7 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v/>
+        <v>Challenge 27</v>
       </c>
       <c r="B122" t="str">
         <v>Route 121</v>
@@ -2843,7 +2843,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v/>
+        <v>Challenge 27</v>
       </c>
       <c r="B123" t="str">
         <v>Route 121</v>
@@ -2863,7 +2863,7 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v/>
+        <v>Challenge 27</v>
       </c>
       <c r="B124" t="str">
         <v>Route 121</v>
@@ -2883,7 +2883,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v/>
+        <v>Challenge 27</v>
       </c>
       <c r="B125" t="str">
         <v>Route 121</v>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B126" t="str">
         <v>Safari Zone East</v>
@@ -2923,7 +2923,7 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B127" t="str">
         <v>Safari Zone East</v>
@@ -2943,7 +2943,7 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B128" t="str">
         <v>Safari Zone East</v>
@@ -2963,7 +2963,7 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B129" t="str">
         <v>Safari Zone East</v>
@@ -2983,7 +2983,7 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B130" t="str">
         <v>Safari Zone East</v>
@@ -3003,7 +3003,7 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B131" t="str">
         <v>Safari Zone East</v>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B132" t="str">
         <v>Safari Zone East</v>
@@ -3043,7 +3043,7 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B133" t="str">
         <v>Safari Zone East</v>
@@ -3063,7 +3063,7 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B134" t="str">
         <v>Safari Zone East</v>
@@ -3083,7 +3083,7 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B135" t="str">
         <v>Safari Zone West</v>
@@ -3103,7 +3103,7 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B136" t="str">
         <v>Safari Zone West</v>
@@ -3123,7 +3123,7 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B137" t="str">
         <v>Safari Zone West</v>
@@ -3143,7 +3143,7 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B138" t="str">
         <v>Safari Zone West</v>
@@ -3163,7 +3163,7 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B139" t="str">
         <v>Safari Zone West</v>
@@ -3183,7 +3183,7 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B140" t="str">
         <v>Safari Zone West</v>
@@ -3203,7 +3203,7 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B141" t="str">
         <v>Safari Zone West</v>
@@ -3223,7 +3223,7 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B142" t="str">
         <v>Safari Zone West</v>
@@ -3243,7 +3243,7 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B143" t="str">
         <v>Safari Zone West</v>
@@ -3263,7 +3263,7 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B144" t="str">
         <v>Safari Zone West</v>
@@ -3283,7 +3283,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B145" t="str">
         <v>Safari Zone North</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B146" t="str">
         <v>Safari Zone North</v>
@@ -3323,7 +3323,7 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B147" t="str">
         <v>Safari Zone North</v>
@@ -3343,7 +3343,7 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B148" t="str">
         <v>Safari Zone North</v>
@@ -3363,7 +3363,7 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B149" t="str">
         <v>Safari Zone North</v>
@@ -3383,7 +3383,7 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B150" t="str">
         <v>Safari Zone North</v>
@@ -3403,7 +3403,7 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B151" t="str">
         <v>Safari Zone North</v>
@@ -3423,7 +3423,7 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v/>
+        <v>Challenge 28</v>
       </c>
       <c r="B152" t="str">
         <v>Safari Zone North</v>
@@ -3443,7 +3443,7 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v/>
+        <v>Challenge 29</v>
       </c>
       <c r="B153" t="str">
         <v>Mount Pyre</v>
@@ -3463,7 +3463,7 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v/>
+        <v>Challenge 29</v>
       </c>
       <c r="B154" t="str">
         <v>Mount Pyre</v>
@@ -3483,7 +3483,7 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v/>
+        <v>Challenge 29</v>
       </c>
       <c r="B155" t="str">
         <v>Mount Pyre</v>
@@ -3503,7 +3503,7 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v/>
+        <v>Challenge 29</v>
       </c>
       <c r="B156" t="str">
         <v>Mount Pyre</v>
@@ -3523,7 +3523,7 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v/>
+        <v>Challenge 29</v>
       </c>
       <c r="B157" t="str">
         <v>Mount Pyre</v>
@@ -3543,7 +3543,7 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v/>
+        <v>Challenge 30</v>
       </c>
       <c r="B158" t="str">
         <v>Route 123</v>
@@ -3563,7 +3563,7 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v/>
+        <v>Challenge 30</v>
       </c>
       <c r="B159" t="str">
         <v>Route 123</v>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v/>
+        <v>Challenge 30</v>
       </c>
       <c r="B160" t="str">
         <v>Route 123</v>
@@ -3603,7 +3603,7 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v/>
+        <v>Challenge 30</v>
       </c>
       <c r="B161" t="str">
         <v>Route 123</v>
@@ -3623,7 +3623,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v/>
+        <v>Challenge 30</v>
       </c>
       <c r="B162" t="str">
         <v>Route 123</v>
@@ -3643,7 +3643,7 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B163" t="str">
         <v>Big Fishing Spot</v>
@@ -3663,7 +3663,7 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B164" t="str">
         <v>Big Fishing Spot</v>
@@ -3683,7 +3683,7 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B165" t="str">
         <v>Big Fishing Spot</v>
@@ -3703,7 +3703,7 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B166" t="str">
         <v>Big Fishing Spot</v>
@@ -3723,7 +3723,7 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B167" t="str">
         <v>Big Fishing Spot</v>
@@ -3743,7 +3743,7 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B168" t="str">
         <v>Big Fishing Spot</v>
@@ -3763,7 +3763,7 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v/>
+        <v>Challenge 33</v>
       </c>
       <c r="B169" t="str">
         <v>Big Fishing Spot</v>
@@ -3783,7 +3783,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v/>
+        <v>Challenge 34</v>
       </c>
       <c r="B170" t="str">
         <v>Underwater Fishing Spot</v>
@@ -3803,7 +3803,7 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v/>
+        <v>Challenge 34</v>
       </c>
       <c r="B171" t="str">
         <v>Underwater Fishing Spot</v>
@@ -3823,7 +3823,7 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v/>
+        <v>Challenge 34</v>
       </c>
       <c r="B172" t="str">
         <v>Underwater Fishing Spot</v>
@@ -3843,7 +3843,7 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v/>
+        <v>Challenge 36</v>
       </c>
       <c r="B173" t="str">
         <v>Shoal Cave</v>
@@ -3863,7 +3863,7 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v/>
+        <v>Challenge 36</v>
       </c>
       <c r="B174" t="str">
         <v>Shoal Cave</v>
@@ -3883,7 +3883,7 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v/>
+        <v>Challenge 36</v>
       </c>
       <c r="B175" t="str">
         <v>Shoal Cave</v>
@@ -3903,7 +3903,7 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v/>
+        <v>Challenge 36</v>
       </c>
       <c r="B176" t="str">
         <v>Shoal Cave</v>
@@ -3923,7 +3923,7 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v/>
+        <v>Challenge 37</v>
       </c>
       <c r="B177" t="str">
         <v>Mirage Island</v>
@@ -3943,7 +3943,7 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v/>
+        <v>Challenge 42</v>
       </c>
       <c r="B178" t="str">
         <v>Victory Road</v>
@@ -3963,7 +3963,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v/>
+        <v>Challenge 42</v>
       </c>
       <c r="B179" t="str">
         <v>Victory Road</v>
@@ -3983,7 +3983,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v/>
+        <v>Challenge 42</v>
       </c>
       <c r="B180" t="str">
         <v>Victory Road</v>
@@ -4003,7 +4003,7 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v/>
+        <v>Challenge 42</v>
       </c>
       <c r="B181" t="str">
         <v>Victory Road</v>
@@ -4023,7 +4023,7 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v/>
+        <v>Challenge 42</v>
       </c>
       <c r="B182" t="str">
         <v>Victory Road</v>
@@ -4043,7 +4043,7 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v/>
+        <v>Challenge 42</v>
       </c>
       <c r="B183" t="str">
         <v>Victory Road</v>
@@ -4063,7 +4063,7 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v/>
+        <v>Challenge 41</v>
       </c>
       <c r="B184" t="str">
         <v>Sky Pillar</v>
@@ -4083,7 +4083,7 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v/>
+        <v>Challenge 41</v>
       </c>
       <c r="B185" t="str">
         <v>Sky Pillar</v>
@@ -4103,7 +4103,7 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v/>
+        <v>Challenge 41</v>
       </c>
       <c r="B186" t="str">
         <v>Sky Pillar</v>
@@ -4123,7 +4123,7 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v/>
+        <v>Challenge 41</v>
       </c>
       <c r="B187" t="str">
         <v>Sky Pillar</v>
@@ -4143,7 +4143,7 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v/>
+        <v>Challenge 41</v>
       </c>
       <c r="B188" t="str">
         <v>Sky Pillar</v>
@@ -4163,7 +4163,7 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v/>
+        <v>Key to Nebula Fissure Challenge</v>
       </c>
       <c r="B189" t="str">
         <v>Nebula Fissure</v>
@@ -4183,7 +4183,7 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v/>
+        <v>Key to Nebula Fissure Challenge</v>
       </c>
       <c r="B190" t="str">
         <v>Nebula Fissure</v>
@@ -4203,7 +4203,7 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v/>
+        <v>Key to Nebula Fissure Challenge</v>
       </c>
       <c r="B191" t="str">
         <v>Nebula Fissure</v>
@@ -4223,7 +4223,7 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v/>
+        <v>Key to Nebula Fissure Challenge</v>
       </c>
       <c r="B192" t="str">
         <v>Nebula Fissure</v>
@@ -4243,7 +4243,7 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B193" t="str">
         <v>Trick House</v>
@@ -4263,7 +4263,7 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B194" t="str">
         <v>Trick House</v>
@@ -4283,7 +4283,7 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B195" t="str">
         <v>Trick House</v>
@@ -4303,7 +4303,7 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B196" t="str">
         <v>Trick House</v>
@@ -4323,7 +4323,7 @@
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v/>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B197" t="str">
         <v>Rustboro Fossil Lab</v>
@@ -4343,7 +4343,7 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v/>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B198" t="str">
         <v>Rustboro Fossil Lab</v>
@@ -4363,7 +4363,7 @@
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v/>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B199" t="str">
         <v>Rustboro Fossil Lab</v>
@@ -4383,7 +4383,7 @@
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v/>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B200" t="str">
         <v>Rustboro Fossil Lab</v>
@@ -4403,7 +4403,7 @@
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v/>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B201" t="str">
         <v>Abandoned Ship</v>
@@ -4423,7 +4423,7 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v/>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B202" t="str">
         <v>Abandoned Ship</v>
@@ -4443,7 +4443,7 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v/>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B203" t="str">
         <v>Abandoned Ship</v>
@@ -4463,7 +4463,7 @@
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v/>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B204" t="str">
         <v>Abandoned Ship</v>
@@ -4483,7 +4483,7 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v/>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B205" t="str">
         <v>Enemy Hideout</v>
@@ -4503,7 +4503,7 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v/>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B206" t="str">
         <v>Enemy Hideout</v>
@@ -4523,7 +4523,7 @@
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v/>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B207" t="str">
         <v>Enemy Hideout</v>
@@ -4543,7 +4543,7 @@
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v/>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B208" t="str">
         <v>Enemy Hideout</v>
@@ -4563,7 +4563,7 @@
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v/>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B209" t="str">
         <v>Sealed Chamber</v>
@@ -4583,7 +4583,7 @@
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v/>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B210" t="str">
         <v>Sealed Chamber</v>
@@ -4603,7 +4603,7 @@
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v/>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B211" t="str">
         <v>Sealed Chamber</v>
@@ -4623,7 +4623,7 @@
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v/>
+        <v>Extra Challenge B 5</v>
       </c>
       <c r="B212" t="str">
         <v>Ancient Ruins</v>
@@ -4643,7 +4643,7 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v/>
+        <v>Extra Challenge B 5</v>
       </c>
       <c r="B213" t="str">
         <v>Ancient Ruins</v>
@@ -4663,7 +4663,7 @@
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v/>
+        <v>Extra Challenge B 5</v>
       </c>
       <c r="B214" t="str">
         <v>Ancient Ruins</v>
@@ -4683,7 +4683,7 @@
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B215" t="str">
         <v>Mauville Game Corner</v>
@@ -4703,7 +4703,7 @@
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B216" t="str">
         <v>Mauville Game Corner</v>
@@ -4723,7 +4723,7 @@
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B217" t="str">
         <v>Mauville Game Corner</v>
@@ -4743,7 +4743,7 @@
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B218" t="str">
         <v>Mauville Game Corner</v>
@@ -4763,7 +4763,7 @@
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v/>
+        <v>Extra Challenge A 1</v>
       </c>
       <c r="B219" t="str">
         <v>Starter Sanctuary</v>
@@ -4783,7 +4783,7 @@
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v/>
+        <v>Extra Challenge A 1</v>
       </c>
       <c r="B220" t="str">
         <v>Starter Sanctuary</v>
@@ -4803,7 +4803,7 @@
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v/>
+        <v>Extra Challenge A 1</v>
       </c>
       <c r="B221" t="str">
         <v>Starter Sanctuary</v>
@@ -4823,7 +4823,7 @@
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v/>
+        <v>Extra Challenge A 2</v>
       </c>
       <c r="B222" t="str">
         <v>Daycare Special Spot</v>
@@ -4843,7 +4843,7 @@
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v/>
+        <v>Extra Challenge A 2</v>
       </c>
       <c r="B223" t="str">
         <v>Daycare Special Spot</v>
@@ -4863,7 +4863,7 @@
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v/>
+        <v>Extra Challenge A 2</v>
       </c>
       <c r="B224" t="str">
         <v>Daycare Special Spot</v>
@@ -4883,7 +4883,7 @@
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v/>
+        <v>Extra Challenge A 2</v>
       </c>
       <c r="B225" t="str">
         <v>Daycare Special Spot</v>
@@ -4903,7 +4903,7 @@
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v/>
+        <v>Extra Challenge A 3</v>
       </c>
       <c r="B226" t="str">
         <v>Battle Frontier Facility</v>
@@ -4923,7 +4923,7 @@
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v/>
+        <v>Extra Challenge A 3</v>
       </c>
       <c r="B227" t="str">
         <v>Battle Frontier Facility</v>
@@ -4943,7 +4943,7 @@
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v/>
+        <v>Extra Challenge A 3</v>
       </c>
       <c r="B228" t="str">
         <v>Battle Frontier Facility</v>
@@ -4963,7 +4963,7 @@
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v/>
+        <v>Extra Challenge A 3</v>
       </c>
       <c r="B229" t="str">
         <v>Battle Frontier Facility</v>
@@ -4983,7 +4983,7 @@
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v/>
+        <v>Extra Challenge A 4</v>
       </c>
       <c r="B230" t="str">
         <v>Weather Climax Cave</v>
@@ -5003,7 +5003,7 @@
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v/>
+        <v>Extra Challenge A 4</v>
       </c>
       <c r="B231" t="str">
         <v>Weather Climax Cave</v>
@@ -5023,7 +5023,7 @@
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v/>
+        <v>Extra Challenge A 4</v>
       </c>
       <c r="B232" t="str">
         <v>Weather Climax Cave</v>
@@ -5043,7 +5043,7 @@
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B233" t="str">
         <v>Roaming Hoenn Skies</v>
@@ -5063,7 +5063,7 @@
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v/>
+        <v>Challenge 44</v>
       </c>
       <c r="B234" t="str">
         <v>Roaming Hoenn Skies</v>
@@ -5090,10 +5090,627 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:C56"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Challenge Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Requisite</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Reward</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Challenge 1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Catch 2 Poochyena</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Unlocks: Route 103</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Challenge 2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Catch 1 Wingull</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Unlocks: Route 102</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Challenge 3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Catch 1 Lotad, Catch 1 Seedot</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Unlocks: Route 104</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Challenge 4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Catch 2 Taillow</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Unlocks: Petalburg Woods</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Challenge 5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Catch 1 Shroomish, Catch 1 Slakoth</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Unlocks: Route 116; Gift: 1 Bug Stone</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Challenge 6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Catch 2 Whismur</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Unlocks: Rustboro Gym</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Challenge 7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Earn Stone Badge</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Unlocks: Granite Cave</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Challenge 8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Catch 1 Makuhita, Catch 1 Aron</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Unlocks: Tiny Fishing Spot; Gift: 1 Rock Stone</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Challenge 9</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v>Unlocks: Dewford Gym</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Challenge 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Earn Knuckle Badge</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Unlocks: Route 107</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Challenge 11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Defeat 50 on Route 107</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Unlocks: Mauville Gym</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Challenge 12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Earn Dynamo Badge</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Unlocks: Route 110</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Challenge 13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Catch 2 Electrike, Catch 1 Plusle, Catch 1 Minun</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Unlocks: Route 117</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Challenge 14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Catch 1 Illumise, Catch 1 Volbeat</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Unlocks: Route 111</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Challenge 15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Catch 1 Trapinch, Catch 1 Cacnea</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Unlocks: Lavaridge Gym</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Challenge 16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Earn Heat Badge</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Unlocks: Fiery Path</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Challenge 17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Catch 2 Numel, Catch 1 Torkoal</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Unlocks: Jagged Pass; Gift: 1 Fire Stone</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Challenge 18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Defeat 100 on Jagged Pass</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Unlocks: Route 113</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Challenge 19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Catch 5 Spinda</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Unlocks: Route 114</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Challenge 20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Catch 1 Zangoose, Catch 1 Seviper</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Unlocks: Meteor Falls</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Challenge 21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Catch 1 Bagon, Catch 1 Solrock, Catch 1 Lunatone</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Unlocks: Route 115; Gift: 1 Dragon Stone</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Challenge 22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Catch 2 Swablu</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Unlocks: Petalburg Gym</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Challenge 23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Earn Balance Badge</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Unlocks: Route 118</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Challenge 24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Catch 1 Manectric, Catch 1 Kecleon</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Unlocks: Small Fishing Spot</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Challenge 25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Catch 1 Carvanha, Catch 1 Barboach</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Unlocks: Route 119</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Challenge 26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Catch 2 Tropius</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Unlocks: Route 120</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Challenge 27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Catch 1 Absol</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Unlocks: Route 121</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Challenge 28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Catch 2 Shuppet, Catch 2 Duskull</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Unlocks: Safari Zone East, Safari Zone West, Safari Zone North</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Challenge 29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Defeat 150 on Safari Zone East</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Unlocks: Mount Pyre</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Challenge 30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Catch 1 Chimecho</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Unlocks: Route 123; Gift: 2 Ghost Stone</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Challenge 31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Defeat 150 on Route 123</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Unlocks: Fortree Gym</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Challenge 32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Earn Feather Badge</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Unlocks: Mossdeep Gym</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Challenge 33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Earn Mind Badge</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Unlocks: Big Fishing Spot</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Challenge 34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Catch 1 Feebas, Catch 2 Wailmer</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Unlocks: Underwater Fishing Spot; Gift: 2 Water Stone</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Challenge 35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Catch 1 Relicanth, Catch 2 Clamperl</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Unlocks: Sootopolis Gym</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Challenge 36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Earn Rain Badge</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Unlocks: Shoal Cave</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Challenge 37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Catch 2 Spheal, Catch 1 Snorunt</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Unlocks: Mirage Island; Gift: 1 Ice Stone</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Challenge 41</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Catch 1 Wynaut</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Unlocks: Sky Pillar</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Challenge 42</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Catch 1 Altaria, Catch 1 Claydol</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Unlocks: Victory Road</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Challenge 43</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Defeat 200 on Victory Road</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Unlocks: Hoenn Pokemon League</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Challenge 44</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Defeat Hoenn Champion</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Unlocks: Roaming Hoenn Skies, Mauville Game Corner, Trick House; Gifts: 2 Masterball</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Extra Challenge A 1</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Catch 8 Common (Slakoth/Abra)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Unlocks: Starter Sanctuary; Gift: 3 Fire Stone</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Extra Challenge A 2</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Catch 1 Treecko, Catch 1 Torchic, Catch 1 Mudkip</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Unlocks: Daycare Special Spot; Gift: 3 Leaf Stone</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Extra Challenge A 3</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Catch 1 Wynaut, Catch 1 Azurill</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Unlocks: Battle Frontier Facility; Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Extra Challenge A 4</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Defeat 50 on Battle Frontier Facility</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Unlocks: Weather Climax Cave; Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Extra Challenge A 5</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Catch 1 Kyogre, Catch 1 Groudon, Catch 1 Rayquaza</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Unlocks: Key to Nebula Fissure Challenge; Gift: 2 Masterball</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Extra Challenge B 1</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Defeat 20 on Trick House</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Unlocks: Rustboro Fossil Lab; Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Extra Challenge B 2</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Catch 1 Lileep, Catch 1 Anorith</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Unlocks: Abandoned Ship; Gift: 1 Root Fossil</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Extra Challenge B 3</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Catch 1 Tentacruel</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Unlocks: Enemy Hideout; Gift: 1 Deep Sea Scale</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Extra Challenge B 4</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Catch 1 Weezing; Defeat 25 on Enemy Hideout</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Unlocks: Sealed Chamber; Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Extra Challenge B 5</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Defeat 1 Relicanth</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Unlocks: Ancient Ruins; Gift: 2 Masterball</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Extra Challenge B 6</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Catch 1 Regirock, Catch 1 Regice, Catch 1 Registeel</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Unlocks: Key to Nebula Fissure Challenge; Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Extra Challenge (Roaming)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Defeat 1 Latias, Defeat 1 Latios</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Unlocks: Key to Nebula Fissure Challenge; Gift: 1 Masterball</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Key to Nebula Fissure Challenge</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Complete challenges: Extra Challenge A 5, Extra Challenge B 6, Extra Challenge (Roaming)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Unlocks: Nebula Fissure</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Nebula Fissure Challenge</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Defeat 1 Deoxys</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Gift: 1 Masterball</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C56"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: generate consolidated 3_Hoenn_Data.xlsx with 4 sheets
- Consolidates Region 3 routing documentation into a single 4-sheet `.xlsx` file.
- Sheet 1: Routes and Spawns mapped to Unlocks
- Sheet 2: Challenge Requirements and Rewards
- Sheet 3: Missing/Evolvable Regional Pokémon
- Sheet 4: Complete Map Coordinate Checklist
- Replaces obsolete isolated Region3Spots file.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/3_Hoenn_Data.xlsx
+++ b/3_Hoenn_Data.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -6475,4 +6476,554 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B45"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C49"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name of challenge</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Route Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Map?</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v>Route 101</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Challenge 1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Route 103</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Challenge 2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Route 102</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Challenge 3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Route 104</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Challenge 4</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Petalburg Woods</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Challenge 5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Route 116</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Challenge 7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Granite Cave</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Challenge 8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tiny Fishing Spot</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Challenge 10</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Route 107</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Challenge 12</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Route 110</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Challenge 13</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Route 117</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Challenge 14</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Route 111</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Challenge 16</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Fiery Path</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Challenge 17</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Jagged Pass</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Challenge 18</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Route 113</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Challenge 19</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Route 114</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Challenge 20</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Meteor Falls</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Challenge 21</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Route 115</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Challenge 23</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Route 118</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Challenge 24</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Small Fishing Spot</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Challenge 25</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Route 119</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Challenge 26</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Route 120</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Challenge 27</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Route 121</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Challenge 28</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Safari Zone East</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Challenge 28</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Safari Zone West</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Challenge 28</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Safari Zone North</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Challenge 29</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Mount Pyre</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Challenge 30</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Route 123</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Challenge 33</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Big Fishing Spot</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Challenge 34</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Underwater Fishing Spot</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Challenge 36</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Shoal Cave</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Challenge 37</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Mirage Island</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Challenge 42</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Victory Road</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Challenge 41</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Sky Pillar</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Key to Nebula Fissure Challenge</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Nebula Fissure</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Challenge 44</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Trick House</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Extra Challenge B 1</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Rustboro Fossil Lab</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Extra Challenge B 2</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Abandoned Ship</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Extra Challenge B 3</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Enemy Hideout</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Extra Challenge B 4</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Sealed Chamber</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Extra Challenge B 5</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Ancient Ruins</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Challenge 44</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Mauville Game Corner</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Extra Challenge A 1</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Starter Sanctuary</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Extra Challenge A 3</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Daycare Special Spot</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Extra Challenge A 4</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Battle Frontier Facility</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Extra Challenge A 5</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Weather Climax Cave</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Challenge 44</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Roaming Hoenn Skies</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Extra Challenge A 2</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Advanced Starter Sanctuary</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update Safari Zone and Hoenn routing data
- Updates level caps and spawns across Safari Zone East, West, and North.
- Distributes missing Pokémon perfectly aligned with type-logic across remaining Hoenn maps.
- Scales Extra Challenge chains to strictly reach level 100+ caps before encountering Legendaries.
- Updates documentation generation to output a 4-sheet consolidated `3_Hoenn_Data.xlsx` replacing separate files.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/3_Hoenn_Data.xlsx
+++ b/3_Hoenn_Data.xlsx
@@ -3156,7 +3156,7 @@
         <v>Pinsir</v>
       </c>
       <c r="E138" t="str">
-        <v>46-50</v>
+        <v>51-55</v>
       </c>
       <c r="F138" t="str">
         <v>8.00%</v>
@@ -3256,7 +3256,7 @@
         <v>Sunkern</v>
       </c>
       <c r="E143" t="str">
-        <v>46-50</v>
+        <v>44-48</v>
       </c>
       <c r="F143" t="str">
         <v>15.00%</v>
@@ -3276,7 +3276,7 @@
         <v>Shuckle</v>
       </c>
       <c r="E144" t="str">
-        <v>46-50</v>
+        <v>51-55</v>
       </c>
       <c r="F144" t="str">
         <v>10.00%</v>
@@ -3296,7 +3296,7 @@
         <v>Doduo</v>
       </c>
       <c r="E145" t="str">
-        <v>1-1</v>
+        <v>46-50</v>
       </c>
       <c r="F145" t="str">
         <v>12.00%</v>
@@ -3316,7 +3316,7 @@
         <v>Rhyhorn</v>
       </c>
       <c r="E146" t="str">
-        <v>1-1</v>
+        <v>46-50</v>
       </c>
       <c r="F146" t="str">
         <v>8.00%</v>
@@ -3336,7 +3336,7 @@
         <v>Girafarig</v>
       </c>
       <c r="E147" t="str">
-        <v>1-1</v>
+        <v>50-54</v>
       </c>
       <c r="F147" t="str">
         <v>8.00%</v>
@@ -3356,7 +3356,7 @@
         <v>Psyduck</v>
       </c>
       <c r="E148" t="str">
-        <v>1-1</v>
+        <v>46-50</v>
       </c>
       <c r="F148" t="str">
         <v>12.00%</v>
@@ -3376,7 +3376,7 @@
         <v>Xatu</v>
       </c>
       <c r="E149" t="str">
-        <v>1-1</v>
+        <v>50-54</v>
       </c>
       <c r="F149" t="str">
         <v>12.00%</v>
@@ -3396,7 +3396,7 @@
         <v>Teddiursa</v>
       </c>
       <c r="E150" t="str">
-        <v>1-1</v>
+        <v>46-50</v>
       </c>
       <c r="F150" t="str">
         <v>8.00%</v>
@@ -3416,7 +3416,7 @@
         <v>Stantler</v>
       </c>
       <c r="E151" t="str">
-        <v>1-1</v>
+        <v>50-54</v>
       </c>
       <c r="F151" t="str">
         <v>10.00%</v>
@@ -3436,7 +3436,7 @@
         <v>Wooper</v>
       </c>
       <c r="E152" t="str">
-        <v>1-1</v>
+        <v>44-48</v>
       </c>
       <c r="F152" t="str">
         <v>10.00%</v>
@@ -3456,7 +3456,7 @@
         <v>Ledyba</v>
       </c>
       <c r="E153" t="str">
-        <v>1-1</v>
+        <v>44-48</v>
       </c>
       <c r="F153" t="str">
         <v>11.00%</v>
@@ -3476,7 +3476,7 @@
         <v>Gloom</v>
       </c>
       <c r="E154" t="str">
-        <v>1-1</v>
+        <v>48-52</v>
       </c>
       <c r="F154" t="str">
         <v>9.00%</v>
@@ -3496,7 +3496,7 @@
         <v>Heracross</v>
       </c>
       <c r="E155" t="str">
-        <v>1-1</v>
+        <v>51-55</v>
       </c>
       <c r="F155" t="str">
         <v>16.00%</v>
@@ -3516,7 +3516,7 @@
         <v>Wobbuffet</v>
       </c>
       <c r="E156" t="str">
-        <v>1-1</v>
+        <v>48-52</v>
       </c>
       <c r="F156" t="str">
         <v>16.00%</v>
@@ -3536,7 +3536,7 @@
         <v>Golduck</v>
       </c>
       <c r="E157" t="str">
-        <v>1-1</v>
+        <v>51-55</v>
       </c>
       <c r="F157" t="str">
         <v>12.00%</v>
@@ -3556,7 +3556,7 @@
         <v>Mareep</v>
       </c>
       <c r="E158" t="str">
-        <v>1-1</v>
+        <v>44-48</v>
       </c>
       <c r="F158" t="str">
         <v>12.00%</v>
@@ -3576,7 +3576,7 @@
         <v>Gligar</v>
       </c>
       <c r="E159" t="str">
-        <v>1-1</v>
+        <v>48-52</v>
       </c>
       <c r="F159" t="str">
         <v>13.00%</v>
@@ -3596,7 +3596,7 @@
         <v>Pineco</v>
       </c>
       <c r="E160" t="str">
-        <v>1-1</v>
+        <v>44-48</v>
       </c>
       <c r="F160" t="str">
         <v>9.00%</v>
@@ -3616,7 +3616,7 @@
         <v>Quagsire</v>
       </c>
       <c r="E161" t="str">
-        <v>1-1</v>
+        <v>48-52</v>
       </c>
       <c r="F161" t="str">
         <v>13.00%</v>
@@ -3636,7 +3636,7 @@
         <v>Spinarak</v>
       </c>
       <c r="E162" t="str">
-        <v>1-1</v>
+        <v>44-48</v>
       </c>
       <c r="F162" t="str">
         <v>9.00%</v>

</xml_diff>